<commit_message>
Revised Dashboard Formatting Issues
</commit_message>
<xml_diff>
--- a/Guerrero_Maryland_Chart.xlsx
+++ b/Guerrero_Maryland_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EF7538-B2D5-4437-9A10-0B40B02BD241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17328B21-6430-4151-9E33-A52E47D4A0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="772" yWindow="195" windowWidth="20191" windowHeight="12780" firstSheet="1" activeTab="1" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
+    <workbookView xWindow="772" yWindow="0" windowWidth="20191" windowHeight="12780" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="9" r:id="rId1"/>
@@ -33,11 +33,11 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId8"/>
-    <pivotCache cacheId="6" r:id="rId9"/>
-    <pivotCache cacheId="7" r:id="rId10"/>
-    <pivotCache cacheId="8" r:id="rId11"/>
-    <pivotCache cacheId="9" r:id="rId12"/>
+    <pivotCache cacheId="0" r:id="rId8"/>
+    <pivotCache cacheId="1" r:id="rId9"/>
+    <pivotCache cacheId="2" r:id="rId10"/>
+    <pivotCache cacheId="3" r:id="rId11"/>
+    <pivotCache cacheId="4" r:id="rId12"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -37631,6 +37631,15 @@
             </a:rPr>
             <a:t>All other categories showed positive growth throughout the years.</a:t>
           </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1100" baseline="0">
@@ -37694,9 +37703,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>380999</xdr:colOff>
+      <xdr:colOff>552449</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>119062</xdr:rowOff>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7134226" cy="5603585"/>
     <xdr:sp macro="" textlink="">
@@ -37712,7 +37721,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6210299" y="300037"/>
+          <a:off x="6381749" y="266700"/>
           <a:ext cx="7134226" cy="5603585"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -40625,7 +40634,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E37ECCF1-1971-4A76-8B0A-C83B416E6428}" name="PivotTable3" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="19" rowHeaderCaption="Month">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E37ECCF1-1971-4A76-8B0A-C83B416E6428}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="19" rowHeaderCaption="Month">
   <location ref="D2:E51" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" numFmtId="165" showAll="0">
@@ -40933,7 +40942,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A627FA6A-DB9D-4E95-839D-915ADDD7E80C}" name="PivotTable6" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="22" rowHeaderCaption="Category">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A627FA6A-DB9D-4E95-839D-915ADDD7E80C}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="22" rowHeaderCaption="Category">
   <location ref="G12:H19" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField numFmtId="14" showAll="0"/>
@@ -41026,7 +41035,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{590AE81B-2CD4-4220-AE06-25736A26C0E9}" name="PivotTable5" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Category">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{590AE81B-2CD4-4220-AE06-25736A26C0E9}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Category">
   <location ref="G2:J9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField numFmtId="14" showAll="0"/>
@@ -41123,7 +41132,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2B144F28-594C-45A1-A68B-6AF74BE51B59}" name="PivotTable15" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="55" rowHeaderCaption="City Location">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2B144F28-594C-45A1-A68B-6AF74BE51B59}" name="PivotTable15" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="55" rowHeaderCaption="City Location">
   <location ref="A12:C22" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField showAll="0"/>
@@ -42156,7 +42165,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{05FEAB13-95F2-4A66-AE83-743573EEF6F6}" name="PivotTable12" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="36" rowHeaderCaption="Products">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{05FEAB13-95F2-4A66-AE83-743573EEF6F6}" name="PivotTable12" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="36" rowHeaderCaption="Products">
   <location ref="A13:C24" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField showAll="0"/>
@@ -42310,7 +42319,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6039BD4E-587C-4232-A032-7EB82533DEAC}" name="PivotTable13" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Year" colHeaderCaption="Sum of Annual_Revenue">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6039BD4E-587C-4232-A032-7EB82533DEAC}" name="PivotTable13" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Year" colHeaderCaption="Sum of Annual_Revenue">
   <location ref="G2:N8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">

</xml_diff>

<commit_message>
Fixed New Formatting Issue for Executive Report Sheet
</commit_message>
<xml_diff>
--- a/Guerrero_Maryland_Chart.xlsx
+++ b/Guerrero_Maryland_Chart.xlsx
@@ -8,42 +8,43 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17328B21-6430-4151-9E33-A52E47D4A0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0ADBDF7-3930-48A4-8E9B-18FDE1CE5E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="772" yWindow="0" windowWidth="20191" windowHeight="12780" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="9" r:id="rId1"/>
     <sheet name="Executive Report" sheetId="11" r:id="rId2"/>
-    <sheet name="Data_Q2" sheetId="4" r:id="rId3"/>
-    <sheet name="Data_Q4" sheetId="2" r:id="rId4"/>
-    <sheet name="Data_Q5" sheetId="5" r:id="rId5"/>
-    <sheet name="Data_Q6A" sheetId="6" r:id="rId6"/>
-    <sheet name="Data_Q6B" sheetId="8" r:id="rId7"/>
+    <sheet name="KPI Metrics" sheetId="12" r:id="rId3"/>
+    <sheet name="Data_Q2" sheetId="4" r:id="rId4"/>
+    <sheet name="Data_Q4" sheetId="2" r:id="rId5"/>
+    <sheet name="Data_Q5" sheetId="5" r:id="rId6"/>
+    <sheet name="Data_Q6A" sheetId="6" r:id="rId7"/>
+    <sheet name="Data_Q6B" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="D7\">Dashboard!$E$26</definedName>
-    <definedName name="ExternalData_1" localSheetId="3" hidden="1">Data_Q4!$A$1:$E$201</definedName>
-    <definedName name="ExternalData_2" localSheetId="2" hidden="1">Data_Q2!$A$1:$B$49</definedName>
-    <definedName name="ExternalData_3" localSheetId="4" hidden="1">Data_Q5!$A$1:$F$10</definedName>
-    <definedName name="ExternalData_4" localSheetId="5" hidden="1">Data_Q6A!$A$1:$E$11</definedName>
-    <definedName name="ExternalData_5" localSheetId="6" hidden="1">Data_Q6B!$A$1:$E$25</definedName>
+    <definedName name="ExternalData_1" localSheetId="4" hidden="1">Data_Q4!$A$1:$E$201</definedName>
+    <definedName name="ExternalData_2" localSheetId="3" hidden="1">Data_Q2!$A$1:$B$49</definedName>
+    <definedName name="ExternalData_3" localSheetId="5" hidden="1">Data_Q5!$A$1:$F$10</definedName>
+    <definedName name="ExternalData_4" localSheetId="6" hidden="1">Data_Q6A!$A$1:$E$11</definedName>
+    <definedName name="ExternalData_5" localSheetId="7" hidden="1">Data_Q6B!$A$1:$E$25</definedName>
     <definedName name="Slicer_Product_Category">#N/A</definedName>
     <definedName name="Slicer_Years__Revenue_Month">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId8"/>
-    <pivotCache cacheId="1" r:id="rId9"/>
-    <pivotCache cacheId="2" r:id="rId10"/>
-    <pivotCache cacheId="3" r:id="rId11"/>
-    <pivotCache cacheId="4" r:id="rId12"/>
+    <pivotCache cacheId="0" r:id="rId9"/>
+    <pivotCache cacheId="1" r:id="rId10"/>
+    <pivotCache cacheId="2" r:id="rId11"/>
+    <pivotCache cacheId="3" r:id="rId12"/>
+    <pivotCache cacheId="4" r:id="rId13"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
       <x14:slicerCaches>
-        <x14:slicerCache r:id="rId13"/>
         <x14:slicerCache r:id="rId14"/>
+        <x14:slicerCache r:id="rId15"/>
       </x14:slicerCaches>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
@@ -37201,6 +37202,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>71437</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>147638</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>974583</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>174288</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93EE99CF-0CE4-45AE-B9CB-102407D9B365}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
@@ -37307,17 +37351,17 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>300039</xdr:colOff>
+      <xdr:colOff>238123</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>100013</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5700712" cy="5603585"/>
+    <xdr:ext cx="8586789" cy="4742452"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
+        <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47291A87-3805-29B4-4D47-9D7DF285608D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1FE5D9D-61B7-4FCF-86FE-C020DD506B50}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -37325,8 +37369,343 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="300039" y="280988"/>
-          <a:ext cx="5700712" cy="5603585"/>
+          <a:off x="238123" y="276225"/>
+          <a:ext cx="8586789" cy="4742452"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="1E2235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Recommendations:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>For the next quarter, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="1">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Technology</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="1" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> &amp; Accessories </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>should be Manager Reddy's priority investment leading at $5M with a consistent year-over-year growth. In 2025 alone, this category saw a spike of $521,971 with an average transaction size of $454, indicating strong customer willingness to spend on premium products. To leverage this, I strongly suggest introducing bundling promotions for products that bring in the most revenue overall, but with lower transaction counts such as the MSI Creator Z16 to help raise counts. More pricing analysis on highest-demand products like the Lenovo IdeaPad Flex is recommended before making any pricing adjustments to avoid disrupting current demand.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Another category with potential worth exploring </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="1" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>is Stationery &amp; Supplies</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>. While revenue sits at only $102, 807, it is the top 2 in transaction volume with 9,862 transactions  and an average of $10 per transaction. This suggests that customer demand is there, but they are spending minimally for this category. I recommend bundling products in this category with similar categories such as Books (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>General) or Art Supplies to target a student consumer base as a back-to-school or premium studying bundle. This can improve average transaction size across all three categories, and therefore revenue across the board.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Reddy should manage the associated risks that the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Textbook</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> category is showing. Although the category brings in the second highest revenue at $1.5M, data shows an overall decline. Over four years, year-over-year revenue has declined twice, once in 2023 and again in 2025. Although 2024 saw a small recovery of $1,491, it was overshadowed by a deeper decline of $99,322 the following year. Instead of eliminating the category entirely, I recommend shifting to demand-based stocking or exploring a consolidation with the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Books (General) category to reduce inventory risk while maintaining EmporiUm's</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> student customers. </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100">
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Management should prioritize </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>closing the performance gap across stores in Maryland. North Harford drives $8.7M of Maryland's total revenue, driven by transaction count rather than average transaction size. Harford is a significant outlier, with most stores falling </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>within the $288k to $320k range, and Germantown as </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>a</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> secondary outlier at $584,676. Annapolis is the</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> lowest performer. I recommend management investigate Harford's sales tactics or other factors that contribute to its disproportionate success and implement findings across the territory. Mid-tier</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> stores may benefit most from</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>bundle promotions and targeted local marketing campaigns. For Annapolis, a dual improvement plan should be implemented targeting improved staff training and seasonal promotions to drive foot traffic, while also conducting further research into external</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0">
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t> limiting factors outside of management's control such as location or city population.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>238124</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6029325" cy="4570225"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39FF1829-F57D-44E1-9ADF-0B05F2658032}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="238124" y="266700"/>
+          <a:ext cx="6029325" cy="4570225"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -37641,391 +38020,6 @@
             <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
           </a:endParaRPr>
         </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>552449</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="7134226" cy="5603585"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1FE5D9D-61B7-4FCF-86FE-C020DD506B50}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6381749" y="266700"/>
-          <a:ext cx="7134226" cy="5603585"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="1E2235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
-          <a:spAutoFit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Recommendations:</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" b="1">
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>For the next quarter, </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" i="1">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Technology</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" i="1" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> &amp; Accessories </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>should be Manager Reddy's priority investment leading at $5M with a consistent year-over-year growth. In 2025 alone, this category saw a spike of $521,971 with an average transaction size of $454, indicating strong customer willingness to spend on premium products. To leverage this, I strongly suggest introducing bundling promotions for products that bring in the most revenue overall, but with lower transaction counts such as the MSI Creator Z16 to help raise counts. More pricing analysis on highest-demand products like the Lenovo IdeaPad Flex is recommended before making any pricing adjustments to avoid disrupting current demand.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Another category with potential worth exploring </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" i="1" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>is Stationery &amp; Supplies</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>. While revenue sits at only $102, 807, it is the top 2 in transaction volume with 9,862 transactions  and an average of $10 per transaction. This suggests that customer demand is there, but they are spending minimally for this category. I recommend bundling products in this category with similar categories such as Books (</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>General) or Art Supplies to target a student consumer base as a back-to-school or premium studying bundle. This can improve average transaction size across all three categories, and therefore revenue across the board.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Reddy should manage the associated risks that the </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" i="1" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Textbook</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> category is showing. Although the category brings in the second highest revenue at $1.5M, data shows an overall decline. Over four years, year-over-year revenue has declined twice, once in 2023 and again in 2025. Although 2024 saw a small recovery of $1,491, it was overshadowed by a deeper decline of $99,322 the following year. Instead of eliminating the category entirely, I recommend shifting to demand-based stocking or exploring a consolidation with the </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Books (General) category to reduce inventory risk while maintaining EmporiUm's</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> student customers. </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Management should prioritize </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>closing the performance gap across stores in Maryland. North Harford drives $8.7M of Maryland's total revenue, driven by transaction count rather than average transaction size. Harford is a significant outlier, with most stores falling </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>within the $288k to $320k range, and Germantown as </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>a</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> secondary outlier at $584,676. Annapolis is the</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> lowest performer. I recommend management investigate Harford's sales tactics or other factors that contribute to its disproportionate success and implement findings across the territory. Mid-tier</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> stores may benefit most from</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>bundle promotions and targeted local marketing campaigns. For Annapolis, a dual improvement plan should be implemented targeting improved staff training and seasonal promotions to drive foot traffic, while also conducting further research into external</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0">
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> limiting factors outside of management's control such as location or city population.</a:t>
-          </a:r>
-        </a:p>
       </xdr:txBody>
     </xdr:sp>
     <xdr:clientData/>
@@ -38033,7 +38027,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -38152,7 +38146,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -38195,7 +38189,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -38238,7 +38232,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
     <cdr:from>
@@ -38339,7 +38333,7 @@
 </c:userShapes>
 </file>
 
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -38360,49 +38354,6 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{896B2EAE-2DF4-4CCD-8A55-D612CF37155D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks/>
-        </xdr:cNvGraphicFramePr>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>71437</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>147638</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>974583</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>174288</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93EE99CF-0CE4-45AE-B9CB-102407D9B365}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -46679,6 +46630,16 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{715227BC-9D44-4782-9DDA-AEE0F48A8295}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88003D3-AF9C-42C3-A459-CB95A481D3E6}">
   <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -47394,7 +47355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED6BAE6-E998-445C-B735-FDE66E11734B}">
   <dimension ref="A1:J201"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -50980,7 +50941,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AF83DD-F524-4332-83DA-83D4C60BDAAA}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -51323,7 +51284,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F7B6D9B-839E-43F3-9733-2A8CC2EA5496}">
   <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -51663,7 +51624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96188C2-7A45-4A5E-A3F6-4998852103DD}">
   <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
Fixed column widths for Github preview
</commit_message>
<xml_diff>
--- a/Guerrero_Maryland_Chart.xlsx
+++ b/Guerrero_Maryland_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB154A71-6B63-4A31-84B2-D5C444718F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140F2EE5-56A3-49AA-A226-07B59E0A43B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2115" yWindow="23" windowWidth="20355" windowHeight="12862" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
+    <workbookView xWindow="1395" yWindow="450" windowWidth="20355" windowHeight="12780" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="9" r:id="rId1"/>
@@ -15300,7 +15300,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000004-1514-4957-A373-D274C64B9888}"/>
+                <c16:uniqueId val="{00000003-4529-455A-84F6-E879884472B4}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -15340,7 +15340,7 @@
                   <c15:showDataLabelsRange val="0"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000004-1514-4957-A373-D274C64B9888}"/>
+                  <c16:uniqueId val="{00000003-4529-455A-84F6-E879884472B4}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -15441,7 +15441,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-1514-4957-A373-D274C64B9888}"/>
+              <c16:uniqueId val="{00000004-CC05-4A8C-9728-23A6B5EBAAE2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -15527,7 +15527,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-1514-4957-A373-D274C64B9888}"/>
+              <c16:uniqueId val="{00000005-CC05-4A8C-9728-23A6B5EBAAE2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -15613,7 +15613,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000007-1514-4957-A373-D274C64B9888}"/>
+              <c16:uniqueId val="{00000006-CC05-4A8C-9728-23A6B5EBAAE2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -15699,7 +15699,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-1514-4957-A373-D274C64B9888}"/>
+              <c16:uniqueId val="{00000007-CC05-4A8C-9728-23A6B5EBAAE2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -15785,7 +15785,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-1514-4957-A373-D274C64B9888}"/>
+              <c16:uniqueId val="{00000008-CC05-4A8C-9728-23A6B5EBAAE2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -18895,7 +18895,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-36B0-411D-9125-27E1489B19BC}"/>
+                <c16:uniqueId val="{00000003-E9D0-4850-85E8-B5531E1AFB60}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -18935,7 +18935,7 @@
                   <c15:showDataLabelsRange val="0"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000003-36B0-411D-9125-27E1489B19BC}"/>
+                  <c16:uniqueId val="{00000003-E9D0-4850-85E8-B5531E1AFB60}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -19036,7 +19036,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000001F-B5AD-476E-A62C-389AAE0E42A7}"/>
+              <c16:uniqueId val="{00000005-7DB0-41F0-A804-077B8F9C436F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -19122,7 +19122,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000020-B5AD-476E-A62C-389AAE0E42A7}"/>
+              <c16:uniqueId val="{00000006-7DB0-41F0-A804-077B8F9C436F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -19208,7 +19208,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000021-B5AD-476E-A62C-389AAE0E42A7}"/>
+              <c16:uniqueId val="{00000007-7DB0-41F0-A804-077B8F9C436F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -19294,7 +19294,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000022-B5AD-476E-A62C-389AAE0E42A7}"/>
+              <c16:uniqueId val="{00000008-7DB0-41F0-A804-077B8F9C436F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -19380,7 +19380,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000023-B5AD-476E-A62C-389AAE0E42A7}"/>
+              <c16:uniqueId val="{00000009-7DB0-41F0-A804-077B8F9C436F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -37209,13 +37209,13 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>71437</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>147638</xdr:rowOff>
+      <xdr:rowOff>147639</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>974583</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>174288</xdr:rowOff>
+      <xdr:colOff>862012</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>4764</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -46644,7 +46644,8 @@
   <dimension ref="A1:E51"/>
   <sheetFormatPr defaultColWidth="13.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="5" max="5" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.59765625" customWidth="1"/>
+    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -46655,7 +46656,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="12">
         <v>44562</v>
       </c>
@@ -51633,12 +51634,11 @@
     <col min="5" max="5" width="16.796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="20.59765625" customWidth="1"/>
     <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.53125" customWidth="1"/>
+    <col min="11" max="12" width="20.59765625" customWidth="1"/>
     <col min="13" max="13" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.6640625" customWidth="1"/>
+    <col min="14" max="14" width="20.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.45">
@@ -51878,7 +51878,7 @@
         <v>3406262.5999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="24">
         <v>2024</v>
       </c>

</xml_diff>

<commit_message>
Download Excel File for Proper Viewing
</commit_message>
<xml_diff>
--- a/Guerrero_Maryland_Chart.xlsx
+++ b/Guerrero_Maryland_Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/sguerrero_my_yearupunited_org/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{2E787AF6-D30C-44F0-A14F-845EA95831BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2687366A-EC80-4952-B2F3-41392F76CF2E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A3D4AF-A485-4524-977C-602912B55ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2977" yWindow="1688" windowWidth="20521" windowHeight="12780" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
+    <workbookView xWindow="2573" yWindow="322" windowWidth="20520" windowHeight="12780" xr2:uid="{C104094F-8F30-45F4-97A0-6B063CB87B83}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="9" r:id="rId1"/>
@@ -1653,7 +1653,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q2!PivotTable3</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q2!PivotTable3</c:name>
     <c:fmtId val="13"/>
   </c:pivotSource>
   <c:chart>
@@ -2495,7 +2495,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q5!PivotTable15</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q5!PivotTable15</c:name>
     <c:fmtId val="54"/>
   </c:pivotSource>
   <c:chart>
@@ -9129,7 +9129,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q6A!PivotTable12</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q6A!PivotTable12</c:name>
     <c:fmtId val="35"/>
   </c:pivotSource>
   <c:chart>
@@ -11154,7 +11154,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q6B!PivotTable13</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q6B!PivotTable13</c:name>
     <c:fmtId val="13"/>
   </c:pivotSource>
   <c:chart>
@@ -16025,7 +16025,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q6B!PivotTable13</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q6B!PivotTable13</c:name>
     <c:fmtId val="11"/>
   </c:pivotSource>
   <c:chart>
@@ -19620,7 +19620,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q6A!PivotTable12</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q6A!PivotTable12</c:name>
     <c:fmtId val="32"/>
   </c:pivotSource>
   <c:chart>
@@ -21257,7 +21257,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q5!PivotTable15</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q5!PivotTable15</c:name>
     <c:fmtId val="52"/>
   </c:pivotSource>
   <c:chart>
@@ -25891,7 +25891,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q4!PivotTable6</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q4!PivotTable6</c:name>
     <c:fmtId val="19"/>
   </c:pivotSource>
   <c:chart>
@@ -26596,7 +26596,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q2!PivotTable3</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q2!PivotTable3</c:name>
     <c:fmtId val="15"/>
   </c:pivotSource>
   <c:chart>
@@ -27556,7 +27556,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q2!PivotTable3</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q2!PivotTable3</c:name>
     <c:fmtId val="17"/>
   </c:pivotSource>
   <c:chart>
@@ -28516,7 +28516,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q2!PivotTable3</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q2!PivotTable3</c:name>
     <c:fmtId val="18"/>
   </c:pivotSource>
   <c:chart>
@@ -29476,7 +29476,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Guerrero_Maryland_Chart (1).xlsx]Data_Q4!PivotTable6</c:name>
+    <c:name>[Guerrero_Maryland_Chart.xlsx]Data_Q4!PivotTable6</c:name>
     <c:fmtId val="21"/>
   </c:pivotSource>
   <c:chart>
@@ -37209,13 +37209,13 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>71437</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>147639</xdr:rowOff>
+      <xdr:rowOff>147638</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>862012</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>4764</xdr:rowOff>
+      <xdr:colOff>757238</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -38108,15 +38108,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>238125</xdr:colOff>
+      <xdr:colOff>238126</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>100013</xdr:rowOff>
+      <xdr:rowOff>100012</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>263405</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>126663</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>314326</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -46642,11 +46642,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88003D3-AF9C-42C3-A459-CB95A481D3E6}">
   <dimension ref="A1:E51"/>
-  <sheetFormatPr defaultColWidth="13.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="4" max="4" width="20.59765625" customWidth="1"/>
-    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultColWidth="20.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
@@ -51634,7 +51630,7 @@
     <col min="5" max="5" width="16.796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.59765625" customWidth="1"/>
+    <col min="9" max="9" width="25.59765625" customWidth="1"/>
     <col min="10" max="10" width="21" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="20.59765625" customWidth="1"/>
     <col min="13" max="13" width="19.59765625" bestFit="1" customWidth="1"/>

</xml_diff>